<commit_message>
DataDrivenEmployeeWorkflowTest: 10 test scenarios (valid + invalid + edge cases) - all passing
- Implemented invalid data handling with try-catch (Option B)
- Edge case handling: long names, calendar issues, malformed dates
- Updated PersonalDetailsPage.clickDateOfBirthIcon() with JS click
- Updated AddEmployeePage.clickSaveAndWaitForNavigation() with JS click
- Updated ExcelUtil and supporting page objects
- All 10 tests passing: 5 valid + 3 invalid + 2 edge cases
</commit_message>
<xml_diff>
--- a/src/test/resources/employeeData.xlsx
+++ b/src/test/resources/employeeData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kumarv\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://escribasoftware-my.sharepoint.com/personal/vinay_kumar_escriba_de/Documents/Documents/GitHub/selenium-scratch/src/test/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9DB81E5C-8280-4A12-B208-0B3960D14FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="8_{9DB81E5C-8280-4A12-B208-0B3960D14FC0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{727263BE-1522-4346-8D2C-AD7C9AEF364B}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="2" xr2:uid="{02F12093-8BDF-447A-A9D6-6592012A5206}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="53">
   <si>
     <t>firstName</t>
   </si>
@@ -109,9 +109,6 @@
     <t>Johnson</t>
   </si>
   <si>
-    <t>Divorced</t>
-  </si>
-  <si>
     <t>robert.j@test.com</t>
   </si>
   <si>
@@ -151,9 +148,6 @@
     <t>Anderson</t>
   </si>
   <si>
-    <t>invalid-date</t>
-  </si>
-  <si>
     <t>sarah@test.com</t>
   </si>
   <si>
@@ -173,6 +167,39 @@
   </si>
   <si>
     <t>edge@test.com</t>
+  </si>
+  <si>
+    <t>2020-12-31</t>
+  </si>
+  <si>
+    <t>invalid date</t>
+  </si>
+  <si>
+    <t>1993-04-12</t>
+  </si>
+  <si>
+    <t>1986-06-25</t>
+  </si>
+  <si>
+    <t>1990-05-15</t>
+  </si>
+  <si>
+    <t>1992-08-22</t>
+  </si>
+  <si>
+    <t>1988-03-10</t>
+  </si>
+  <si>
+    <t>1995-11-30</t>
+  </si>
+  <si>
+    <t>1991-07-18</t>
+  </si>
+  <si>
+    <t>Other</t>
+  </si>
+  <si>
+    <t>1985-06-03</t>
   </si>
 </sst>
 </file>
@@ -225,7 +252,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -233,19 +260,23 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -588,7 +619,8 @@
   <cols>
     <col min="1" max="1" width="29.42578125" style="1" customWidth="1"/>
     <col min="2" max="2" width="30.5703125" style="1" customWidth="1"/>
-    <col min="3" max="4" width="28.28515625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="28.28515625" style="9" customWidth="1"/>
+    <col min="4" max="4" width="28.28515625" style="1" customWidth="1"/>
     <col min="5" max="5" width="30.42578125" style="1" customWidth="1"/>
     <col min="6" max="6" width="33.140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="32" style="1" customWidth="1"/>
@@ -603,7 +635,7 @@
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="9" t="s">
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
@@ -629,8 +661,8 @@
       <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="5">
-        <v>33008</v>
+      <c r="C2" s="9" t="s">
+        <v>46</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>11</v>
@@ -641,7 +673,7 @@
       <c r="F2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="4" t="s">
         <v>14</v>
       </c>
       <c r="H2" s="1">
@@ -655,8 +687,8 @@
       <c r="B3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="5">
-        <v>33838</v>
+      <c r="C3" s="9" t="s">
+        <v>47</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>11</v>
@@ -667,7 +699,7 @@
       <c r="F3" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="4" t="s">
         <v>19</v>
       </c>
       <c r="H3" s="1">
@@ -681,20 +713,20 @@
       <c r="B4" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="5">
-        <v>32212</v>
+      <c r="C4" s="9" t="s">
+        <v>48</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>11</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>22</v>
+        <v>51</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G4" s="6" t="s">
-        <v>23</v>
+      <c r="G4" s="4" t="s">
+        <v>22</v>
       </c>
       <c r="H4" s="1">
         <v>9876543212</v>
@@ -702,13 +734,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="B5" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B5" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C5" s="5">
-        <v>35033</v>
+      <c r="C5" s="9" t="s">
+        <v>49</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>11</v>
@@ -719,8 +751,8 @@
       <c r="F5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="G5" s="6" t="s">
-        <v>26</v>
+      <c r="G5" s="4" t="s">
+        <v>25</v>
       </c>
       <c r="H5" s="1">
         <v>9876543213</v>
@@ -728,13 +760,13 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="C6" s="5">
-        <v>33437</v>
+      <c r="C6" s="9" t="s">
+        <v>50</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>11</v>
@@ -745,8 +777,8 @@
       <c r="F6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="G6" s="6" t="s">
-        <v>29</v>
+      <c r="G6" s="4" t="s">
+        <v>28</v>
       </c>
       <c r="H6" s="1">
         <v>9876543214</v>
@@ -769,43 +801,43 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="10.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.42578125" style="8" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="5" t="s">
         <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" s="3">
-        <v>34071</v>
+        <v>29</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>44</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>11</v>
@@ -816,8 +848,8 @@
       <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>31</v>
+      <c r="G2" s="3" t="s">
+        <v>30</v>
       </c>
       <c r="H2" s="2">
         <v>9876543215</v>
@@ -825,11 +857,11 @@
     </row>
     <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B3" s="2"/>
-      <c r="C3" s="3">
-        <v>32684</v>
+      <c r="C3" s="7" t="s">
+        <v>45</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>11</v>
@@ -840,8 +872,8 @@
       <c r="F3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>33</v>
+      <c r="G3" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="H3" s="2">
         <v>9876543216</v>
@@ -849,13 +881,13 @@
     </row>
     <row r="4" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B4" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B4" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>36</v>
+      <c r="C4" s="7" t="s">
+        <v>43</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>11</v>
@@ -866,8 +898,8 @@
       <c r="F4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G4" s="4" t="s">
-        <v>37</v>
+      <c r="G4" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="H4" s="2">
         <v>9876543217</v>
@@ -890,7 +922,7 @@
   <cols>
     <col min="1" max="1" width="15.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14.28515625" customWidth="1"/>
-    <col min="3" max="3" width="11.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.42578125" style="8" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.140625" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="7.42578125" bestFit="1" customWidth="1"/>
@@ -898,41 +930,41 @@
     <col min="8" max="8" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="E1" s="7" t="s">
+      <c r="E1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="F1" s="7" t="s">
+      <c r="F1" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="H1" s="5" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C2" s="3">
-        <v>18264</v>
+        <v>37</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>52</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>11</v>
@@ -943,22 +975,22 @@
       <c r="F2" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>40</v>
+      <c r="G2" s="3" t="s">
+        <v>38</v>
       </c>
       <c r="H2" s="2">
         <v>9876543218</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C3" s="7" t="s">
         <v>42</v>
-      </c>
-      <c r="C3" s="3">
-        <v>44196</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>11</v>
@@ -969,8 +1001,8 @@
       <c r="F3" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>43</v>
+      <c r="G3" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="H3" s="2">
         <v>9999999999</v>

</xml_diff>